<commit_message>
pond_jour + chronic diseases
</commit_message>
<xml_diff>
--- a/output/Tables/Modal shift/HIA_modal_shift_1000replicate.xlsx
+++ b/output/Tables/Modal shift/HIA_modal_shift_1000replicate.xlsx
@@ -1,108 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10119"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ines/Documents/PhD/PROJETS/MARCHE/HIA_walking_steps/output/Tables/Modal shift/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EC463D9-89CA-9B41-91F6-DBF9CAE04131}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="500" windowWidth="16100" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
-  <si>
-    <t>disease</t>
-  </si>
-  <si>
-    <t>tot_cases</t>
-  </si>
-  <si>
-    <t>tot_cases_low</t>
-  </si>
-  <si>
-    <t>tot_cases_up</t>
-  </si>
-  <si>
-    <t>tot_daly</t>
-  </si>
-  <si>
-    <t>tot_daly_low</t>
-  </si>
-  <si>
-    <t>tot_daly_up</t>
-  </si>
-  <si>
-    <t>tot_medic_costs</t>
-  </si>
-  <si>
-    <t>tot_medic_costs_low</t>
-  </si>
-  <si>
-    <t>tot_medic_costs_up</t>
-  </si>
-  <si>
-    <t>tot_soc_costs</t>
-  </si>
-  <si>
-    <t>tot_soc_costs_low</t>
-  </si>
-  <si>
-    <t>tot_soc_costs_up</t>
-  </si>
-  <si>
-    <t>mort</t>
-  </si>
-  <si>
-    <t>cvd</t>
-  </si>
-  <si>
-    <t>cancer</t>
-  </si>
-  <si>
-    <t>diab2</t>
-  </si>
-  <si>
-    <t>dem</t>
-  </si>
-  <si>
-    <t>dep</t>
-  </si>
-  <si>
-    <t>Morbidity</t>
-  </si>
-  <si>
-    <t>All</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -150,21 +63,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -202,7 +107,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -236,7 +141,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -271,10 +175,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -447,83 +350,100 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:M9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="2" max="2" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.83203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.83203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.1640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.33203125" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>13</v>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>disease</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>tot_cases</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>tot_cases_low</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>tot_cases_up</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>tot_daly</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>tot_daly_low</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>tot_daly_up</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>tot_medic_costs</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>tot_medic_costs_low</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>tot_medic_costs_up</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>tot_soc_costs</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>tot_soc_costs_low</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>tot_soc_costs_up</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>mort</t>
+        </is>
       </c>
       <c r="B2">
-        <v>70260.221999999994</v>
+        <v>66446.52499999999</v>
       </c>
       <c r="C2">
-        <v>66839.964999999997</v>
+        <v>63098.954</v>
       </c>
       <c r="D2">
-        <v>73733.47</v>
+        <v>69835.985</v>
       </c>
       <c r="E2">
-        <v>721697.35400000005</v>
+        <v>681322.1629999999</v>
       </c>
       <c r="F2">
-        <v>701749.25399999996</v>
+        <v>661729.159</v>
       </c>
       <c r="G2">
-        <v>741853.598</v>
+        <v>701005.789</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -535,200 +455,210 @@
         <v>0</v>
       </c>
       <c r="K2">
-        <v>95987464634.645004</v>
+        <v>90614110421.61</v>
       </c>
       <c r="L2">
-        <v>93321277608.865997</v>
+        <v>88013980902.996</v>
       </c>
       <c r="M2">
-        <v>98669601429.259003</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>14</v>
+        <v>93236846395.505</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>cvd</t>
+        </is>
       </c>
       <c r="B3">
-        <v>49984.754999999997</v>
+        <v>46158.983</v>
       </c>
       <c r="C3">
-        <v>47909.553</v>
+        <v>44176.584</v>
       </c>
       <c r="D3">
-        <v>52072.542999999998</v>
+        <v>48154.461</v>
       </c>
       <c r="E3">
-        <v>44514.578000000001</v>
+        <v>63334.634</v>
       </c>
       <c r="F3">
-        <v>42883.608999999997</v>
+        <v>60896.167</v>
       </c>
       <c r="G3">
-        <v>46161.146000000001</v>
+        <v>65804.67</v>
       </c>
       <c r="H3">
-        <v>2784145627.7950001</v>
+        <v>2432232293.036</v>
       </c>
       <c r="I3">
-        <v>2669448027.5640001</v>
+        <v>2328484218.334</v>
       </c>
       <c r="J3">
-        <v>2900844361.3730001</v>
+        <v>2538040738.695</v>
       </c>
       <c r="K3">
-        <v>5920537410.0249996</v>
+        <v>8424549791.907</v>
       </c>
       <c r="L3">
-        <v>5704047167.0129995</v>
+        <v>8098912074.935</v>
       </c>
       <c r="M3">
-        <v>6139271854.8599997</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>15</v>
+        <v>8750544872.274</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>cancer</t>
+        </is>
       </c>
       <c r="B4">
-        <v>39862.819000000003</v>
+        <v>10756.799</v>
       </c>
       <c r="C4">
-        <v>38155.057999999997</v>
+        <v>10216.652</v>
       </c>
       <c r="D4">
-        <v>41645.54</v>
+        <v>11310.961</v>
       </c>
       <c r="E4">
-        <v>60143.258000000002</v>
+        <v>5055.081</v>
       </c>
       <c r="F4">
-        <v>56929.584000000003</v>
+        <v>4818.466</v>
       </c>
       <c r="G4">
-        <v>63529.945</v>
+        <v>5299.073</v>
       </c>
       <c r="H4">
-        <v>590301912.05400002</v>
+        <v>315421857.623</v>
       </c>
       <c r="I4">
-        <v>564946582.20899999</v>
+        <v>299597857.047</v>
       </c>
       <c r="J4">
-        <v>616730584.48300004</v>
+        <v>331708905.034</v>
       </c>
       <c r="K4">
-        <v>7998322532.3000002</v>
+        <v>672335373.605</v>
       </c>
       <c r="L4">
-        <v>7575713037.7530003</v>
+        <v>640910300.631</v>
       </c>
       <c r="M4">
-        <v>8446470737.2720003</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>16</v>
+        <v>704547780.618</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>diab2</t>
+        </is>
       </c>
       <c r="B5">
-        <v>8147.4870000000001</v>
+        <v>7408.642</v>
       </c>
       <c r="C5">
-        <v>7782.8490000000002</v>
+        <v>7095.962</v>
       </c>
       <c r="D5">
-        <v>8517.8700000000008</v>
+        <v>7729.613</v>
       </c>
       <c r="E5">
-        <v>15903.828</v>
+        <v>13499.944</v>
       </c>
       <c r="F5">
-        <v>15159.56</v>
+        <v>12893.365</v>
       </c>
       <c r="G5">
-        <v>16660.239000000001</v>
+        <v>14123.658</v>
       </c>
       <c r="H5">
-        <v>612629014.36399996</v>
+        <v>290418581.44</v>
       </c>
       <c r="I5">
-        <v>585296207.85599995</v>
+        <v>278201619.036</v>
       </c>
       <c r="J5">
-        <v>640545143.77100003</v>
+        <v>302968364.419</v>
       </c>
       <c r="K5">
-        <v>2114873938.0139999</v>
+        <v>1795421191.616</v>
       </c>
       <c r="L5">
-        <v>2015940343.0190001</v>
+        <v>1714588585.072</v>
       </c>
       <c r="M5">
-        <v>2216145255.823</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>17</v>
+        <v>1878287528.298</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>dem</t>
+        </is>
       </c>
       <c r="B6">
-        <v>17395.733</v>
+        <v>15636.15</v>
       </c>
       <c r="C6">
-        <v>16372.674999999999</v>
+        <v>14690.668</v>
       </c>
       <c r="D6">
-        <v>18435.812000000002</v>
+        <v>16598.535</v>
       </c>
       <c r="E6">
-        <v>28772.697</v>
+        <v>17829.668</v>
       </c>
       <c r="F6">
-        <v>27434.328000000001</v>
+        <v>16736.238</v>
       </c>
       <c r="G6">
-        <v>30128.328000000001</v>
+        <v>18954.774</v>
       </c>
       <c r="H6">
-        <v>292841250.34500003</v>
+        <v>260236094.72</v>
       </c>
       <c r="I6">
-        <v>275756213.16500002</v>
+        <v>244660366.998</v>
       </c>
       <c r="J6">
-        <v>310201915.84899998</v>
+        <v>276172876.875</v>
       </c>
       <c r="K6">
-        <v>3826289156.6880002</v>
+        <v>2371099488.14</v>
       </c>
       <c r="L6">
-        <v>3647639911.6100001</v>
+        <v>2224787528.735</v>
       </c>
       <c r="M6">
-        <v>4007473453.9920001</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>18</v>
+        <v>2521004659.216</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>dep</t>
+        </is>
       </c>
       <c r="B7">
-        <v>159354.56400000001</v>
+        <v>163182.242</v>
       </c>
       <c r="C7">
-        <v>153824.63200000001</v>
+        <v>157405.469</v>
       </c>
       <c r="D7">
-        <v>164980.43400000001</v>
+        <v>168988.283</v>
       </c>
       <c r="E7">
-        <v>51671.99</v>
+        <v>61005.645</v>
       </c>
       <c r="F7">
-        <v>49208.512999999999</v>
+        <v>58202.454</v>
       </c>
       <c r="G7">
-        <v>54217.087</v>
+        <v>63839.351</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -740,95 +670,99 @@
         <v>0</v>
       </c>
       <c r="K7">
-        <v>6872861983.7749996</v>
+        <v>8114227207.434</v>
       </c>
       <c r="L7">
-        <v>6543556287.3649998</v>
+        <v>7739526530.264</v>
       </c>
       <c r="M7">
-        <v>7212584245.0050001</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>19</v>
+        <v>8493792425.47</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Chronic diseases</t>
+        </is>
       </c>
       <c r="B8">
-        <v>274745.35800000001</v>
+        <v>79960.57399999999</v>
       </c>
       <c r="C8">
-        <v>264044.76699999999</v>
+        <v>76179.86600000001</v>
       </c>
       <c r="D8">
-        <v>285652.19900000002</v>
+        <v>83793.57000000001</v>
       </c>
       <c r="E8">
-        <v>201006.351</v>
+        <v>99719.327</v>
       </c>
       <c r="F8">
-        <v>191615.59400000001</v>
+        <v>95344.236</v>
       </c>
       <c r="G8">
-        <v>210696.745</v>
+        <v>104182.175</v>
       </c>
       <c r="H8">
-        <v>4279917804.5580001</v>
+        <v>3298308826.819</v>
       </c>
       <c r="I8">
-        <v>4095447030.7940001</v>
+        <v>3150944061.415</v>
       </c>
       <c r="J8">
-        <v>4468322005.4759998</v>
+        <v>3448890885.023</v>
       </c>
       <c r="K8">
-        <v>26732885020.801998</v>
+        <v>13263405845.268</v>
       </c>
       <c r="L8">
-        <v>25486896746.759998</v>
+        <v>12679198489.373</v>
       </c>
       <c r="M8">
-        <v>28021945546.952</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>20</v>
+        <v>13854384840.406</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
       </c>
       <c r="B9">
-        <v>345005.58</v>
+        <v>309589.341</v>
       </c>
       <c r="C9">
-        <v>330884.73200000002</v>
+        <v>296684.289</v>
       </c>
       <c r="D9">
-        <v>359385.66899999999</v>
+        <v>322617.838</v>
       </c>
       <c r="E9">
-        <v>922703.70500000007</v>
+        <v>842047.1349999999</v>
       </c>
       <c r="F9">
-        <v>893364.848</v>
+        <v>815275.849</v>
       </c>
       <c r="G9">
-        <v>952550.34299999988</v>
+        <v>869027.3150000001</v>
       </c>
       <c r="H9">
-        <v>4279917804.5580001</v>
+        <v>3298308826.819</v>
       </c>
       <c r="I9">
-        <v>4095447030.7940001</v>
+        <v>3150944061.415</v>
       </c>
       <c r="J9">
-        <v>4468322005.4759998</v>
+        <v>3448890885.023</v>
       </c>
       <c r="K9">
-        <v>122720349655.44701</v>
+        <v>111991743474.312</v>
       </c>
       <c r="L9">
-        <v>118808174355.62601</v>
+        <v>108432705922.633</v>
       </c>
       <c r="M9">
-        <v>126691546976.211</v>
+        <v>115585023661.381</v>
       </c>
     </row>
   </sheetData>

</xml_diff>